<commit_message>
Update FMG DOI and server paths
Fix typo and update the FMG DOI to the USF Digital Commons.
Update metadata and input file paths to reflect the current server locations.
</commit_message>
<xml_diff>
--- a/Multibeam_metadata.xlsx
+++ b/Multibeam_metadata.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>comit_wrk/ailich/2015_12/QimeraProjects/2015_12/Export/BAGS/EL1.bag</t>
+          <t>WRK/ailich/2015_12/QimeraProjects/2015_12/Export/BAGS/EL1.bag</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -559,7 +559,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Secondary version projection is UTM 17N event hough should have been UTM 16N</t>
+          <t>Secondary version projection is UTM 17N even though should have been UTM 16N</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>comit_wrk/ailich/2015_12/FMGT_PROJECTS/EL1.fmproj/Output/Mosaic/EL_1_BS_TS_43-47_1m/EL_1_BS_TS_43-47_1m.tif</t>
+          <t>WRK/ailich/2015_12/FMGT_PROJECTS/EL1.fmproj/Output/Mosaic/EL_1_BS_TS_43-47_1m/EL_1_BS_TS_43-47_1m.tif</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>comit_wrk/ailich/2016_05/QimeraProject/2016-05-BEL/Export/BAGS/SWFMG1.bag</t>
+          <t>WRK/ailich/2016_05/QimeraProject/2016-05-BEL/Export/BAGS/SWFMG1.bag</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>comit_wrk/ailich/2016_05/FMGT_Projects/SWFMG1.fmproj/Output/Mosaic/SWFMG_1_BS_TS_43-47_1m/SWFMG_1_BS_TS_43-47_1m.tif</t>
+          <t>WRK/ailich/2016_05/FMGT_Projects/SWFMG1.fmproj/Output/Mosaic/SWFMG_1_BS_TS_43-47_1m/SWFMG_1_BS_TS_43-47_1m.tif</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>comit_wrk/ailich/2016_06/Qimera_Project/2016-06-WB2/Export/BAGS/SWFMG2.bag</t>
+          <t>WRK/ailich/2016_06/Qimera_Project/2016-06-WB2/Export/BAGS/SWFMG2.bag</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>comit_wrk/ailich/2016_06/FMGT_Projects/SWFMG2.fmproj/Output/Mosaic/SWFMG_2_BS_TS_43-47_1m/SWFMG_2_BS_TS_43-47_1m.tif</t>
+          <t>WRK/ailich/2016_06/FMGT_Projects/SWFMG2.fmproj/Output/Mosaic/SWFMG_2_BS_TS_43-47_1m/SWFMG_2_BS_TS_43-47_1m.tif</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>comit_wrk/ailich/2016-07/QimeraProjects/2016-07-BEL/Export/BAGS/SWFMG3.bag</t>
+          <t>WRK/ailich/2016-07/QimeraProjects/2016-07-BEL/Export/BAGS/SWFMG3.bag</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>comit_wrk/ailich/2016-07/FMGT_Projects/SWFMG3.fmproj/Output/Mosaic/SWFMG_3_BS_TS_43-47_1m/SWFMG_3_BS_TS_43-47_1m.tif</t>
+          <t>WRK/ailich/2016-07/FMGT_Projects/SWFMG3.fmproj/Output/Mosaic/SWFMG_3_BS_TS_43-47_1m/SWFMG_3_BS_TS_43-47_1m.tif</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -5389,7 +5389,7 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>comit_wrk/crubiano/New Hi-res WFS surfaces/The Edges/2005_08 Corridor_10m.bag</t>
+          <t>WRK/crubiano/New Hi-res WFS surfaces/The Edges/2005_08 Corridor_10m.bag</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
@@ -5498,12 +5498,12 @@
       </c>
       <c r="U58" t="inlineStr">
         <is>
-          <t>https://www.ngdc.noaa.gov/ships/suncoaster/2006_07_FMG_mb.html</t>
+          <t>https://doi.org/10.17632/8f9hgpff48.1</t>
         </is>
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>Mapping spanned from 2000-2006</t>
+          <t>Mapping spanned from 2000-2006, Gappier UTM  version available at NCEI</t>
         </is>
       </c>
     </row>
@@ -10435,7 +10435,7 @@
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>comit_wrk/crubiano/New Hi-res WFS surfaces/Pulley Ridge (Full footprint)/S_Pulley_Ridge_West_10m.bag</t>
+          <t>WRK/crubiano/New Hi-res WFS surfaces/Pulley Ridge (Full footprint)/S_Pulley_Ridge_West_10m.bag</t>
         </is>
       </c>
       <c r="O130" t="inlineStr">

</xml_diff>